<commit_message>
Updated policy scehdules for 4.0.7
</commit_message>
<xml_diff>
--- a/InputData/elec/HYECFCA/HIst Year Elec Cap Fac Cal Adjust.xlsx
+++ b/InputData/elec/HYECFCA/HIst Year Elec Cap Fac Cal Adjust.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\HYECFCA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MaryFrancisSwint\Vensim\eps-southkorea\InputData\elec\HYECFCA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DE4846-ACEE-4A36-8C8F-2120F7B91DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D8BB2F-0427-4831-B4F4-C4F2364B7F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{2434D2BD-6D34-4476-A32C-19CE7C594793}"/>
+    <workbookView xWindow="-38520" yWindow="-3765" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{2434D2BD-6D34-4476-A32C-19CE7C594793}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -560,14 +560,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9E2E221-CC08-48E5-88DE-512F1AA684C0}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -586,96 +586,109 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:AA26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>27</v>
       </c>
       <c r="B1">
+        <v>2021</v>
+      </c>
+      <c r="C1">
+        <v>2022</v>
+      </c>
+      <c r="D1">
+        <v>2023</v>
+      </c>
+      <c r="E1">
+        <v>2024</v>
+      </c>
+      <c r="F1">
         <v>2025</v>
       </c>
-      <c r="C1">
+      <c r="G1">
         <v>2026</v>
       </c>
-      <c r="D1">
+      <c r="H1">
         <v>2027</v>
       </c>
-      <c r="E1">
+      <c r="I1">
         <v>2028</v>
       </c>
-      <c r="F1">
+      <c r="J1">
         <v>2029</v>
       </c>
-      <c r="G1">
+      <c r="K1">
         <v>2030</v>
       </c>
-      <c r="H1">
+      <c r="L1">
         <v>2031</v>
       </c>
-      <c r="I1">
+      <c r="M1">
         <v>2032</v>
       </c>
-      <c r="J1">
+      <c r="N1">
         <v>2033</v>
       </c>
-      <c r="K1">
+      <c r="O1">
         <v>2034</v>
       </c>
-      <c r="L1">
+      <c r="P1">
         <v>2035</v>
       </c>
-      <c r="M1">
+      <c r="Q1">
         <v>2036</v>
       </c>
-      <c r="N1">
+      <c r="R1">
         <v>2037</v>
       </c>
-      <c r="O1">
+      <c r="S1">
         <v>2038</v>
       </c>
-      <c r="P1">
+      <c r="T1">
         <v>2039</v>
       </c>
-      <c r="Q1">
+      <c r="U1">
         <v>2040</v>
       </c>
-      <c r="R1">
+      <c r="V1">
         <v>2041</v>
       </c>
-      <c r="S1">
+      <c r="W1">
         <v>2042</v>
       </c>
-      <c r="T1">
+      <c r="X1">
         <v>2043</v>
       </c>
-      <c r="U1">
+      <c r="Y1">
         <v>2044</v>
       </c>
-      <c r="V1">
+      <c r="Z1">
         <v>2045</v>
       </c>
-      <c r="W1">
+      <c r="AA1">
         <v>2046</v>
       </c>
-      <c r="X1">
+      <c r="AB1">
         <v>2047</v>
       </c>
-      <c r="Y1">
+      <c r="AC1">
         <v>2048</v>
       </c>
-      <c r="Z1">
+      <c r="AD1">
         <v>2049</v>
       </c>
-      <c r="AA1">
+      <c r="AE1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -757,8 +770,20 @@
       <c r="AA2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB2">
+        <v>1</v>
+      </c>
+      <c r="AC2">
+        <v>1</v>
+      </c>
+      <c r="AD2">
+        <v>1</v>
+      </c>
+      <c r="AE2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -840,8 +865,20 @@
       <c r="AA3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB3">
+        <v>1</v>
+      </c>
+      <c r="AC3">
+        <v>1</v>
+      </c>
+      <c r="AD3">
+        <v>1</v>
+      </c>
+      <c r="AE3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -923,8 +960,20 @@
       <c r="AA4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB4">
+        <v>1</v>
+      </c>
+      <c r="AC4">
+        <v>1</v>
+      </c>
+      <c r="AD4">
+        <v>1</v>
+      </c>
+      <c r="AE4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1007,8 +1056,20 @@
       <c r="AA5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB5">
+        <v>1</v>
+      </c>
+      <c r="AC5">
+        <v>1</v>
+      </c>
+      <c r="AD5">
+        <v>1</v>
+      </c>
+      <c r="AE5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1091,8 +1152,20 @@
       <c r="AA6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB6">
+        <v>1</v>
+      </c>
+      <c r="AC6">
+        <v>1</v>
+      </c>
+      <c r="AD6">
+        <v>1</v>
+      </c>
+      <c r="AE6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1175,8 +1248,20 @@
       <c r="AA7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB7">
+        <v>1</v>
+      </c>
+      <c r="AC7">
+        <v>1</v>
+      </c>
+      <c r="AD7">
+        <v>1</v>
+      </c>
+      <c r="AE7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1259,8 +1344,20 @@
       <c r="AA8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB8">
+        <v>1</v>
+      </c>
+      <c r="AC8">
+        <v>1</v>
+      </c>
+      <c r="AD8">
+        <v>1</v>
+      </c>
+      <c r="AE8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1343,8 +1440,20 @@
       <c r="AA9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB9">
+        <v>1</v>
+      </c>
+      <c r="AC9">
+        <v>1</v>
+      </c>
+      <c r="AD9">
+        <v>1</v>
+      </c>
+      <c r="AE9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1427,8 +1536,20 @@
       <c r="AA10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB10">
+        <v>1</v>
+      </c>
+      <c r="AC10">
+        <v>1</v>
+      </c>
+      <c r="AD10">
+        <v>1</v>
+      </c>
+      <c r="AE10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1511,8 +1632,20 @@
       <c r="AA11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB11">
+        <v>1</v>
+      </c>
+      <c r="AC11">
+        <v>1</v>
+      </c>
+      <c r="AD11">
+        <v>1</v>
+      </c>
+      <c r="AE11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1594,8 +1727,20 @@
       <c r="AA12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB12">
+        <v>1</v>
+      </c>
+      <c r="AC12">
+        <v>1</v>
+      </c>
+      <c r="AD12">
+        <v>1</v>
+      </c>
+      <c r="AE12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1677,8 +1822,20 @@
       <c r="AA13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB13">
+        <v>1</v>
+      </c>
+      <c r="AC13">
+        <v>1</v>
+      </c>
+      <c r="AD13">
+        <v>1</v>
+      </c>
+      <c r="AE13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1760,8 +1917,20 @@
       <c r="AA14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB14">
+        <v>1</v>
+      </c>
+      <c r="AC14">
+        <v>1</v>
+      </c>
+      <c r="AD14">
+        <v>1</v>
+      </c>
+      <c r="AE14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1844,8 +2013,20 @@
       <c r="AA15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB15">
+        <v>1</v>
+      </c>
+      <c r="AC15">
+        <v>1</v>
+      </c>
+      <c r="AD15">
+        <v>1</v>
+      </c>
+      <c r="AE15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1927,8 +2108,20 @@
       <c r="AA16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB16">
+        <v>1</v>
+      </c>
+      <c r="AC16">
+        <v>1</v>
+      </c>
+      <c r="AD16">
+        <v>1</v>
+      </c>
+      <c r="AE16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -2010,8 +2203,20 @@
       <c r="AA17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB17">
+        <v>1</v>
+      </c>
+      <c r="AC17">
+        <v>1</v>
+      </c>
+      <c r="AD17">
+        <v>1</v>
+      </c>
+      <c r="AE17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2094,8 +2299,20 @@
       <c r="AA18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB18">
+        <v>1</v>
+      </c>
+      <c r="AC18">
+        <v>1</v>
+      </c>
+      <c r="AD18">
+        <v>1</v>
+      </c>
+      <c r="AE18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2177,8 +2394,20 @@
       <c r="AA19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB19">
+        <v>1</v>
+      </c>
+      <c r="AC19">
+        <v>1</v>
+      </c>
+      <c r="AD19">
+        <v>1</v>
+      </c>
+      <c r="AE19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -2260,8 +2489,20 @@
       <c r="AA20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB20">
+        <v>1</v>
+      </c>
+      <c r="AC20">
+        <v>1</v>
+      </c>
+      <c r="AD20">
+        <v>1</v>
+      </c>
+      <c r="AE20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -2343,8 +2584,20 @@
       <c r="AA21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB21">
+        <v>1</v>
+      </c>
+      <c r="AC21">
+        <v>1</v>
+      </c>
+      <c r="AD21">
+        <v>1</v>
+      </c>
+      <c r="AE21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -2426,8 +2679,20 @@
       <c r="AA22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB22">
+        <v>1</v>
+      </c>
+      <c r="AC22">
+        <v>1</v>
+      </c>
+      <c r="AD22">
+        <v>1</v>
+      </c>
+      <c r="AE22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -2509,8 +2774,20 @@
       <c r="AA23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB23">
+        <v>1</v>
+      </c>
+      <c r="AC23">
+        <v>1</v>
+      </c>
+      <c r="AD23">
+        <v>1</v>
+      </c>
+      <c r="AE23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -2592,8 +2869,20 @@
       <c r="AA24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB24">
+        <v>1</v>
+      </c>
+      <c r="AC24">
+        <v>1</v>
+      </c>
+      <c r="AD24">
+        <v>1</v>
+      </c>
+      <c r="AE24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -2675,8 +2964,20 @@
       <c r="AA25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="AB25">
+        <v>1</v>
+      </c>
+      <c r="AC25">
+        <v>1</v>
+      </c>
+      <c r="AD25">
+        <v>1</v>
+      </c>
+      <c r="AE25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>3</v>
       </c>
@@ -2756,6 +3057,18 @@
         <v>1</v>
       </c>
       <c r="AA26">
+        <v>1</v>
+      </c>
+      <c r="AB26">
+        <v>1</v>
+      </c>
+      <c r="AC26">
+        <v>1</v>
+      </c>
+      <c r="AD26">
+        <v>1</v>
+      </c>
+      <c r="AE26">
         <v>1</v>
       </c>
     </row>
@@ -2767,19 +3080,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0F07B30-2289-4DFA-B2A9-691D5E6D350E}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -2793,7 +3106,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2808,7 +3121,7 @@
         <v>0.99925866186869106</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -2823,7 +3136,7 @@
         <v>0.97656769537997867</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -2838,7 +3151,7 @@
         <v>0.99049996775136739</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -2853,7 +3166,7 @@
         <v>1.0669161325664203</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -2868,7 +3181,7 @@
         <v>0.93648670812995327</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -2883,7 +3196,7 @@
         <v>1.0238947796972699</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -2898,7 +3211,7 @@
         <v>1.0049882422482364</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -2913,7 +3226,7 @@
         <v>1.0687524097695031</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -2928,12 +3241,12 @@
         <v>0.99999935568255771</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
HYECFCA and SoCtICoS updated for SK data
</commit_message>
<xml_diff>
--- a/InputData/elec/HYECFCA/HIst Year Elec Cap Fac Cal Adjust.xlsx
+++ b/InputData/elec/HYECFCA/HIst Year Elec Cap Fac Cal Adjust.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MaryFrancisSwint\Vensim\eps-southkorea\InputData\elec\HYECFCA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D8BB2F-0427-4831-B4F4-C4F2364B7F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B957A870-1BEE-4889-921F-602CA0C5D384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-3765" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{2434D2BD-6D34-4476-A32C-19CE7C594793}"/>
+    <workbookView xWindow="-37260" yWindow="-2505" windowWidth="28800" windowHeight="15225" activeTab="3" xr2:uid="{2434D2BD-6D34-4476-A32C-19CE7C594793}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="HYECFCA" sheetId="2" r:id="rId2"/>
     <sheet name="Calibration 2025" sheetId="3" r:id="rId3"/>
+    <sheet name="Calibration 2021-24" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="60">
   <si>
     <t>HYECFCA Historical Year Electricity Capacity Factor Calibration Adjustment</t>
   </si>
@@ -179,12 +180,57 @@
   </si>
   <si>
     <t>Model 2025 generation, HYECFCA=1 (MWh, from CAL25H0.tab - Vensim exports 6 significant figures)</t>
+  </si>
+  <si>
+    <t>South Korea HYECFCA calibration 2021-24: multiplier so modeled generation matches KESIS observed generation</t>
+  </si>
+  <si>
+    <t>Applies to sources whose modeled output follows the SYSHECF curves (hard coal and nuclear/hydro/wind/solar/MSW). Gas, petroleum are least-cost dispatched (MCF/BDTPTUMCF=1) and are not scaled by HYECFCA. 2025+ stays 1 so the forecast is untouched. Biomass stays 1: observed biomass (11.8-12.1 TWh) includes wood-pellet co-firing and bio heavy oil outside the 972 MW biomass fleet, so no multiplier can reconcile it (model 5.9-6.2 TWh already at ~73% CF).</t>
+  </si>
+  <si>
+    <t>Observed: KESIS / Korea Energy Statistics, copied from InputData/elec/RPSDbS workbook tabs "Power Generation by ES" (nuclear, coal; GWh) and "New n Renewable" (solar, wind, hydro, waste; MWh). Wind observed is onshore+offshore combined, so one factor applies to both. Solar compared against generation including distributed. Model: South Korea develop_4.0.7 BAU (no .cin), Electricity Generation by Type Including Distributed Generation; run H1 = HYECFCA all 1; H3 = final factors after two corrections (first pass obs/model, then residual re-fit because coal dispatch interacts with gas).</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>hard coal</t>
+  </si>
+  <si>
+    <t>KESIS observed generation (TWh)</t>
+  </si>
+  <si>
+    <t>Model generation at HYECFCA = 1 (TWh, run H1)</t>
+  </si>
+  <si>
+    <t>First-pass factor = observed / model</t>
+  </si>
+  <si>
+    <t>Final HYECFCA (iterated; run H3)</t>
+  </si>
+  <si>
+    <t>Model generation at final HYECFCA (TWh, run H3)</t>
+  </si>
+  <si>
+    <t>Error vs observed</t>
+  </si>
+  <si>
+    <t>onshore + offshore wind</t>
+  </si>
+  <si>
+    <t>solar PV (incl distributed)</t>
+  </si>
+  <si>
+    <t>2021-24: KESIS observed generation vs model run at HYECFCA=1, iterated - see 'Calibration 2021-24' tab (added 2026-10-28, replaces the US 2025 calibration that was placed in the 2021 column). All other years: 1 (no adjustment). The old 'Calibration 2025' tab is US EIA-923 data, no longer referenced, kept for provenance only.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -222,9 +268,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,6 +614,11 @@
         <v>0</v>
       </c>
     </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+    </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
@@ -693,16 +745,20 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <f>'Calibration 2021-24'!C9</f>
+        <v>1.02088</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D9</f>
+        <v>0.98705600000000004</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E9</f>
+        <v>0.98299599999999998</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F9</f>
+        <v>0.91386599999999996</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -978,17 +1034,20 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <f>'Calibration 2025'!D5</f>
-        <v>0.99925866186869106</v>
+        <f>'Calibration 2021-24'!C16</f>
+        <v>0.99597199999999997</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D16</f>
+        <v>0.99446599999999996</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E16</f>
+        <v>0.992838</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F16</f>
+        <v>0.97264799999999996</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1074,17 +1133,20 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <f>'Calibration 2025'!D6</f>
-        <v>0.97656769537997867</v>
+        <f>'Calibration 2021-24'!C23</f>
+        <v>0.99849100000000002</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D23</f>
+        <v>1.0169429999999999</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E23</f>
+        <v>1.0193620000000001</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F23</f>
+        <v>1.2817449999999999</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1170,17 +1232,20 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <f>'Calibration 2025'!D7</f>
-        <v>0.99049996775136739</v>
+        <f>'Calibration 2021-24'!C30</f>
+        <v>1.0916429999999999</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D30</f>
+        <v>1.0953660000000001</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E30</f>
+        <v>1.062425</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F30</f>
+        <v>0.983572</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -1266,17 +1331,20 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <f>'Calibration 2025'!D8</f>
-        <v>1.0669161325664203</v>
+        <f>'Calibration 2021-24'!C37</f>
+        <v>1.003622</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D37</f>
+        <v>1.060147</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E37</f>
+        <v>0.98583799999999999</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F37</f>
+        <v>0.96180100000000002</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -1362,8 +1430,7 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <f>'Calibration 2025'!D9</f>
-        <v>0.93648670812995327</v>
+        <v>1</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1458,8 +1525,7 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <f>'Calibration 2025'!D10</f>
-        <v>1.0238947796972699</v>
+        <v>1</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1554,8 +1620,7 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <f>'Calibration 2025'!D11</f>
-        <v>1.0049882422482364</v>
+        <v>1</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1935,17 +2000,20 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <f>'Calibration 2025'!D12</f>
-        <v>1.0687524097695031</v>
+        <f>'Calibration 2021-24'!C30</f>
+        <v>1.0916429999999999</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D30</f>
+        <v>1.0953660000000001</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E30</f>
+        <v>1.062425</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F30</f>
+        <v>0.983572</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -2221,17 +2289,20 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <f>'Calibration 2025'!D13</f>
-        <v>0.99999935568255771</v>
+        <f>'Calibration 2021-24'!C44</f>
+        <v>0.58614999999999995</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <f>'Calibration 2021-24'!D44</f>
+        <v>0.52037500000000003</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <f>'Calibration 2021-24'!E44</f>
+        <v>0.55270799999999998</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <f>'Calibration 2021-24'!F44</f>
+        <v>0.52898699999999999</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -3254,4 +3325,823 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9A0D3B-0E4B-484A-AA31-18AF80276B54}">
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28.6328125" customWidth="1"/>
+    <col min="2" max="2" width="48.6328125" customWidth="1"/>
+    <col min="3" max="6" width="11.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2021</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2022</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2023</v>
+      </c>
+      <c r="F5" s="1">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6">
+        <v>197.96600000000001</v>
+      </c>
+      <c r="D6">
+        <v>193.23099999999999</v>
+      </c>
+      <c r="E6">
+        <v>184.92699999999999</v>
+      </c>
+      <c r="F6">
+        <v>167.15199999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7">
+        <v>193.917</v>
+      </c>
+      <c r="D7">
+        <v>195.77099999999999</v>
+      </c>
+      <c r="E7">
+        <v>187.881</v>
+      </c>
+      <c r="F7">
+        <v>181.756</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8">
+        <f>C6/C7</f>
+        <v>1.0208800672452647</v>
+      </c>
+      <c r="D8">
+        <f>D6/D7</f>
+        <v>0.98702565752843885</v>
+      </c>
+      <c r="E8">
+        <f>E6/E7</f>
+        <v>0.98427728189651953</v>
+      </c>
+      <c r="F8">
+        <f>F6/F7</f>
+        <v>0.91965052047800344</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9">
+        <v>1.02088</v>
+      </c>
+      <c r="D9">
+        <v>0.98705600000000004</v>
+      </c>
+      <c r="E9">
+        <v>0.98299599999999998</v>
+      </c>
+      <c r="F9">
+        <v>0.91386599999999996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10">
+        <v>197.96600000000001</v>
+      </c>
+      <c r="D10">
+        <v>193.22900000000001</v>
+      </c>
+      <c r="E10">
+        <v>184.94399999999999</v>
+      </c>
+      <c r="F10">
+        <v>167.208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2">
+        <f>C10/C6-1</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="2">
+        <f>D10/D6-1</f>
+        <v>-1.0350306110185059E-5</v>
+      </c>
+      <c r="E11" s="2">
+        <f>E10/E6-1</f>
+        <v>9.1928166249255483E-5</v>
+      </c>
+      <c r="F11" s="2">
+        <f>F10/F6-1</f>
+        <v>3.3502440892130281E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13">
+        <v>158.01499999999999</v>
+      </c>
+      <c r="D13">
+        <v>176.054</v>
+      </c>
+      <c r="E13">
+        <v>180.494</v>
+      </c>
+      <c r="F13">
+        <v>188.75399999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14">
+        <v>158.654</v>
+      </c>
+      <c r="D14">
+        <v>177.07499999999999</v>
+      </c>
+      <c r="E14">
+        <v>181.79599999999999</v>
+      </c>
+      <c r="F14">
+        <v>194.06200000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15">
+        <f>C13/C14</f>
+        <v>0.99597236754194651</v>
+      </c>
+      <c r="D15">
+        <f>D13/D14</f>
+        <v>0.9942340816038403</v>
+      </c>
+      <c r="E15">
+        <f>E13/E14</f>
+        <v>0.99283812625140266</v>
+      </c>
+      <c r="F15">
+        <f>F13/F14</f>
+        <v>0.97264791664519579</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16">
+        <v>0.99597199999999997</v>
+      </c>
+      <c r="D16">
+        <v>0.99446599999999996</v>
+      </c>
+      <c r="E16">
+        <v>0.992838</v>
+      </c>
+      <c r="F16">
+        <v>0.97264799999999996</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17">
+        <v>158.01499999999999</v>
+      </c>
+      <c r="D17">
+        <v>176.03399999999999</v>
+      </c>
+      <c r="E17">
+        <v>180.494</v>
+      </c>
+      <c r="F17">
+        <v>188.75399999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="2">
+        <f>C17/C13-1</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="2">
+        <f>D17/D13-1</f>
+        <v>-1.136015086280473E-4</v>
+      </c>
+      <c r="E18" s="2">
+        <f>E17/E13-1</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="2">
+        <f>F17/F13-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20">
+        <v>3.05721</v>
+      </c>
+      <c r="D20">
+        <v>3.5448659999999999</v>
+      </c>
+      <c r="E20">
+        <v>3.7180149999999998</v>
+      </c>
+      <c r="F20">
+        <v>4.3134880000000004</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21">
+        <v>3.0618300000000001</v>
+      </c>
+      <c r="D21">
+        <v>3.48597</v>
+      </c>
+      <c r="E21">
+        <v>3.64744</v>
+      </c>
+      <c r="F21">
+        <v>3.3661500000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22">
+        <f>C20/C21</f>
+        <v>0.99849109846072448</v>
+      </c>
+      <c r="D22">
+        <f>D20/D21</f>
+        <v>1.0168951540030464</v>
+      </c>
+      <c r="E22">
+        <f>E20/E21</f>
+        <v>1.0193491873752549</v>
+      </c>
+      <c r="F22">
+        <f>F20/F21</f>
+        <v>1.2814307146146191</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23">
+        <v>0.99849100000000002</v>
+      </c>
+      <c r="D23">
+        <v>1.0169429999999999</v>
+      </c>
+      <c r="E23">
+        <v>1.0193620000000001</v>
+      </c>
+      <c r="F23">
+        <v>1.2817449999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24">
+        <v>3.05721</v>
+      </c>
+      <c r="D24">
+        <v>3.5448200000000001</v>
+      </c>
+      <c r="E24">
+        <v>3.7180200000000001</v>
+      </c>
+      <c r="F24">
+        <v>4.3134800000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="2">
+        <f>C24/C20-1</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="2">
+        <f>D24/D20-1</f>
+        <v>-1.2976513075413365E-5</v>
+      </c>
+      <c r="E25" s="2">
+        <f>E24/E20-1</f>
+        <v>1.344803611580403E-6</v>
+      </c>
+      <c r="F25" s="2">
+        <f>F24/F20-1</f>
+        <v>-1.8546475614167335E-6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27">
+        <v>3.1800169999999999</v>
+      </c>
+      <c r="D27">
+        <v>3.3694579999999998</v>
+      </c>
+      <c r="E27">
+        <v>3.3921649999999999</v>
+      </c>
+      <c r="F27">
+        <v>3.7365689999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28">
+        <v>2.9147530000000001</v>
+      </c>
+      <c r="D28">
+        <v>3.0779860000000001</v>
+      </c>
+      <c r="E28">
+        <v>3.1940360000000001</v>
+      </c>
+      <c r="F28">
+        <v>3.7986110000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29">
+        <f>C27/C28</f>
+        <v>1.0910073683773547</v>
+      </c>
+      <c r="D29">
+        <f>D27/D28</f>
+        <v>1.0946956873747964</v>
+      </c>
+      <c r="E29">
+        <f>E27/E28</f>
+        <v>1.0620309226320555</v>
+      </c>
+      <c r="F29">
+        <f>F27/F28</f>
+        <v>0.98366718782207485</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30">
+        <v>1.0916429999999999</v>
+      </c>
+      <c r="D30">
+        <v>1.0953660000000001</v>
+      </c>
+      <c r="E30">
+        <v>1.062425</v>
+      </c>
+      <c r="F30">
+        <v>0.983572</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31">
+        <v>3.1800050000000004</v>
+      </c>
+      <c r="D31">
+        <v>3.3694000000000002</v>
+      </c>
+      <c r="E31">
+        <v>3.3921549999999998</v>
+      </c>
+      <c r="F31">
+        <v>3.7365729999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="2">
+        <f>C31/C27-1</f>
+        <v>-3.7735647323566823E-6</v>
+      </c>
+      <c r="D32" s="2">
+        <f>D31/D27-1</f>
+        <v>-1.7213450946629294E-5</v>
+      </c>
+      <c r="E32" s="2">
+        <f>E31/E27-1</f>
+        <v>-2.947969806932349E-6</v>
+      </c>
+      <c r="F32" s="2">
+        <f>F31/F27-1</f>
+        <v>1.0705007722489057E-6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34">
+        <v>24.717623</v>
+      </c>
+      <c r="D34">
+        <v>30.72626</v>
+      </c>
+      <c r="E34">
+        <v>33.236446999999998</v>
+      </c>
+      <c r="F34">
+        <v>37.449731</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" t="s">
+        <v>52</v>
+      </c>
+      <c r="C35">
+        <v>24.639500000000002</v>
+      </c>
+      <c r="D35">
+        <v>29.189800000000002</v>
+      </c>
+      <c r="E35">
+        <v>33.654499999999999</v>
+      </c>
+      <c r="F35">
+        <v>38.741599999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36">
+        <f>C34/C35</f>
+        <v>1.0031706406379999</v>
+      </c>
+      <c r="D36">
+        <f>D34/D35</f>
+        <v>1.0526368800060295</v>
+      </c>
+      <c r="E36">
+        <f>E34/E35</f>
+        <v>0.98757809505415317</v>
+      </c>
+      <c r="F36">
+        <f>F34/F35</f>
+        <v>0.96665421665599771</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37">
+        <v>1.003622</v>
+      </c>
+      <c r="D37">
+        <v>1.060147</v>
+      </c>
+      <c r="E37">
+        <v>0.98583799999999999</v>
+      </c>
+      <c r="F37">
+        <v>0.96180100000000002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38">
+        <v>24.716000000000001</v>
+      </c>
+      <c r="D38">
+        <v>30.696000000000002</v>
+      </c>
+      <c r="E38">
+        <v>33.244700000000002</v>
+      </c>
+      <c r="F38">
+        <v>37.478200000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="2">
+        <f>C38/C34-1</f>
+        <v>-6.5661653630644246E-5</v>
+      </c>
+      <c r="D39" s="2">
+        <f>D38/D34-1</f>
+        <v>-9.8482535785349157E-4</v>
+      </c>
+      <c r="E39" s="2">
+        <f>E38/E34-1</f>
+        <v>2.4831174042172499E-4</v>
+      </c>
+      <c r="F39" s="2">
+        <f>F38/F34-1</f>
+        <v>7.6019237628166536E-4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" t="s">
+        <v>51</v>
+      </c>
+      <c r="C41">
+        <v>0.47061999999999998</v>
+      </c>
+      <c r="D41">
+        <v>0.41352899999999998</v>
+      </c>
+      <c r="E41">
+        <v>0.44376900000000002</v>
+      </c>
+      <c r="F41">
+        <v>0.42472399999999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42">
+        <v>0.80289999999999995</v>
+      </c>
+      <c r="D42">
+        <v>0.79469400000000001</v>
+      </c>
+      <c r="E42">
+        <v>0.80289999999999995</v>
+      </c>
+      <c r="F42">
+        <v>0.80289999999999995</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>53</v>
+      </c>
+      <c r="C43">
+        <f>C41/C42</f>
+        <v>0.58615020550504426</v>
+      </c>
+      <c r="D43">
+        <f>D41/D42</f>
+        <v>0.52036255464367409</v>
+      </c>
+      <c r="E43">
+        <f>E41/E42</f>
+        <v>0.55270768464316855</v>
+      </c>
+      <c r="F43">
+        <f>F41/F42</f>
+        <v>0.52898742060032389</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>41</v>
+      </c>
+      <c r="B44" t="s">
+        <v>54</v>
+      </c>
+      <c r="C44">
+        <v>0.58614999999999995</v>
+      </c>
+      <c r="D44">
+        <v>0.52037500000000003</v>
+      </c>
+      <c r="E44">
+        <v>0.55270799999999998</v>
+      </c>
+      <c r="F44">
+        <v>0.52898699999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45">
+        <v>0.47061999999999998</v>
+      </c>
+      <c r="D45">
+        <v>0.41352</v>
+      </c>
+      <c r="E45">
+        <v>0.44376900000000002</v>
+      </c>
+      <c r="F45">
+        <v>0.42472399999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>41</v>
+      </c>
+      <c r="B46" t="s">
+        <v>56</v>
+      </c>
+      <c r="C46" s="2">
+        <f>C45/C41-1</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="2">
+        <f>D45/D41-1</f>
+        <v>-2.1763890803216945E-5</v>
+      </c>
+      <c r="E46" s="2">
+        <f>E45/E41-1</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="2">
+        <f>F45/F41-1</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>